<commit_message>
Agrega sensibilidad con la tarifa publicada en los folletos
- Simula 0.9% trimestral, 0.1% mensual y 15 UDIS/mes (folletos Allianz
  2023 y 2025, p. 11) con escalas por cargo: EscalasCargosPPR,
  TARIFA_FOLLETO_2025, sim_tarifa_folleto.py, su JSON y la gráfica 07.
- Comparte los topes de la CG 3.12 como constantes; el JSON deriva de
  ellas sus tarifas y una prueba nueva detecta desalineaciones.
- Declara que los folletos (p. 10) describen el bono generado en el
  primer año, mientras el modelo sigue la CG 3.6 ($150/mes).
- README: tabla y gráfica del folleto, diferencias de versión, fuentes,
  validación de PDF descargados y cifras recalculadas (§1, §2, §5.2, §5.4).
- Excel: supuestos del folleto y del bono; rag.py retira una precisión
  no reproducible; .gitignore excluye tmp/.
</commit_message>
<xml_diff>
--- a/outputs/resultados_ppr_vs_vuaa.xlsx
+++ b/outputs/resultados_ppr_vs_vuaa.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -624,12 +624,12 @@
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Cargos PPR (típico)</t>
+          <t>Cargos PPR (mitad)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Mitad de los topes (la carátula puede cobrar menos)</t>
+          <t>Mitad de cada tope; hipótesis, no tarifa publicada</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -641,100 +641,117 @@
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Bono de Fidelidad</t>
+          <t>Cargos PPR (folleto 2025)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>75% de la aportación comprometida del primer año (45,000 en total), generado pro rata (150/mes); rinde inflación+5% (tope 9%) menos cargos; acreditado año 25. Se supone instrucción para reinvertirlo al rendimiento de mercado; CG indica renta fija corta por defecto</t>
+          <t>0.9% trimestral administración + 0.1% mensual gestión + 15 UDIS/mes desde mes 19; no es escenario base del Excel</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>CG Allianz 3.6 y 3.10.3; folleto OptiMaxx plus p.2 y p.5</t>
+          <t>Allianz México, folletos OptiMaxx plus 2023 y 2025 (misma tarifa), p. 11; resultados_tarifa_folleto.json</t>
         </is>
       </c>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ISR salida PPR</t>
+          <t>Bono de Fidelidad</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Caso base: retiro único y toda la exención disponible, hasta 90 UMA elevadas al año (3.85M en 2026, crece con la UMA); tarifa anual sobre el excedente. Otras pensiones pueden consumir la exención; ver sensibilidad fiscal</t>
+          <t>75% de la aportación comprometida del primer año (45,000 en total). Generación repartida entre los 300 pagos comprometidos (150/mes): interpretación del modelo de CG 3.6; los folletos 2023 y 2025 (p. 10) la describen durante el primer año. Rinde inflación+5% (tope 9%) menos cargos; acreditado año 25. Se supone instrucción para reinvertirlo al rendimiento de mercado; CG indica renta fija corta por defecto</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>CG 3.21; regla 3.17.6 RMF; art. 171 RLISR</t>
+          <t>CG Allianz 3.6 y 3.10.3; folletos 2023 y 2025, p. 10, solo para el 75% del primer año</t>
         </is>
       </c>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ISR salida VUAA</t>
+          <t>ISR salida PPR</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>10% definitivo sobre la ganancia; costo de adquisición actualizado por inflación</t>
+          <t>Caso base: retiro único y toda la exención disponible, hasta 90 UMA elevadas al año (3.85M en 2026, crece con la UMA); tarifa anual sobre el excedente. Otras pensiones pueden consumir la exención; ver sensibilidad fiscal</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Art. 129 LISR</t>
+          <t>CG 3.21; regla 3.17.6 RMF; art. 171 RLISR</t>
         </is>
       </c>
     </row>
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Tarifa ISR</t>
+          <t>ISR salida VUAA</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2026 congelada nominalmente 40 años (simplificación; indexarla favorece al PPR 0.1-0.7M)</t>
+          <t>10% definitivo sobre la ganancia; costo de adquisición actualizado por inflación</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Anexo 8 RMF 2026</t>
+          <t>Art. 129 LISR</t>
         </is>
       </c>
     </row>
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>VUAA costos</t>
+          <t>Tarifa ISR</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Corretaje supuesto 0.25% + IVA por operación + OCF 0.07% anual</t>
+          <t>2026 congelada nominalmente 40 años (simplificación; indexarla favorece al PPR 0.1-0.7M)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Vanguard México (OCF 2026); corretaje supuesto</t>
+          <t>Anexo 8 RMF 2026</t>
         </is>
       </c>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>VUAA costos</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Corretaje supuesto 0.25% + IVA por operación + OCF 0.07% anual</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Vanguard México (OCF 2026); corretaje supuesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>UDI / UMA 2026</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>8.826356 MXN / 117.31 MXN diaria</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Banxico / INEGI (sept-2026)</t>
         </is>

</xml_diff>